<commit_message>
Aggiornato il file PCPC.xlsx con nuove misurazioni e risultati
</commit_message>
<xml_diff>
--- a/mpi/lab8/results/PCPC.xlsx
+++ b/mpi/lab8/results/PCPC.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr codeName="Questa_cartella_di_lavoro" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unisalerno-my.sharepoint.com/personal/m_cosenza11_studenti_unisa_it/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\proge\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="746" documentId="8_{95CF893B-CBBC-4BA0-BD94-BC40F482AAA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B671696C-E14B-446F-9277-883F99AC6B18}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{38A27E26-997E-48DA-BA5F-7736BA74A789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{862AEACE-3155-4182-8D10-C10E8BB68475}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{862AEACE-3155-4182-8D10-C10E8BB68475}"/>
   </bookViews>
   <sheets>
     <sheet name="Standard Time" sheetId="5" r:id="rId1"/>
@@ -16702,7 +16702,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="it-IT"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -38593,10 +38593,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="DatiEsterni_1" connectionId="1" xr16:uid="{0DADC74A-6A07-414F-A181-B9E7D5461E96}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
   <queryTableRefresh nextId="10" unboundColumnsRight="3">
@@ -39000,21 +38996,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9390C505-E081-4BA9-AB3C-913B19589443}">
+  <sheetPr codeName="Foglio1"/>
   <dimension ref="A1:AA162"/>
-  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.75" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29.5" customWidth="1"/>
-    <col min="8" max="8" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.44140625" customWidth="1"/>
+    <col min="8" max="8" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -39043,7 +39040,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -39084,7 +39081,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -39125,7 +39122,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -39166,7 +39163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -39207,7 +39204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -39248,7 +39245,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -39289,7 +39286,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -39330,7 +39327,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -39371,7 +39368,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -39412,7 +39409,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -39453,7 +39450,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -39494,7 +39491,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -39535,7 +39532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -39567,7 +39564,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -39599,7 +39596,7 @@
         <v>0.16463414634146342</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -39631,7 +39628,7 @@
         <v>5.4372842347525895E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -39663,7 +39660,7 @@
         <v>1.2711864406779662E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>14</v>
       </c>
@@ -39695,7 +39692,7 @@
         <v>1.0187580853816301E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>14</v>
       </c>
@@ -39727,7 +39724,7 @@
         <v>1.5829145728643218E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>14</v>
       </c>
@@ -39759,7 +39756,7 @@
         <v>6.5190397350993372E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:27" ht="19.05" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:27" ht="18" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -39797,7 +39794,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -39829,7 +39826,7 @@
         <v>5.6566455696202535E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>13</v>
       </c>
@@ -39861,7 +39858,7 @@
         <v>6.3612099644128117E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>13</v>
       </c>
@@ -39893,7 +39890,7 @@
         <v>1.0106235618049312E-4</v>
       </c>
     </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>13</v>
       </c>
@@ -39925,7 +39922,7 @@
         <v>2.9170052840632782E-5</v>
       </c>
     </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>13</v>
       </c>
@@ -39957,7 +39954,7 @@
         <v>1.3641927079606846E-5</v>
       </c>
     </row>
-    <row r="27" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>13</v>
       </c>
@@ -39989,7 +39986,7 @@
         <v>4.4162954507833214E-5</v>
       </c>
     </row>
-    <row r="28" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>13</v>
       </c>
@@ -40021,7 +40018,7 @@
         <v>5.4210725201512258E-6</v>
       </c>
     </row>
-    <row r="29" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>13</v>
       </c>
@@ -40053,7 +40050,7 @@
         <v>2.4448289303616983E-6</v>
       </c>
     </row>
-    <row r="30" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>13</v>
       </c>
@@ -40085,7 +40082,7 @@
         <v>2.1058132580117799E-6</v>
       </c>
     </row>
-    <row r="31" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>13</v>
       </c>
@@ -40117,7 +40114,7 @@
         <v>8.9696420395254869E-7</v>
       </c>
     </row>
-    <row r="32" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>13</v>
       </c>
@@ -40149,7 +40146,7 @@
         <v>5.8176251487522004E-7</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>14</v>
       </c>
@@ -40181,7 +40178,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>14</v>
       </c>
@@ -40213,7 +40210,7 @@
         <v>0.21260683760683763</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>14</v>
       </c>
@@ -40245,7 +40242,7 @@
         <v>3.0096793708408957E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>14</v>
       </c>
@@ -40277,7 +40274,7 @@
         <v>1.3001437344832093E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>14</v>
       </c>
@@ -40309,7 +40306,7 @@
         <v>7.6822112415071038E-3</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>14</v>
       </c>
@@ -40341,7 +40338,7 @@
         <v>5.8051341890315057E-3</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>14</v>
       </c>
@@ -40373,7 +40370,7 @@
         <v>9.8010244286840052E-3</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>13</v>
       </c>
@@ -40405,7 +40402,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>13</v>
       </c>
@@ -40437,7 +40434,7 @@
         <v>0.49043798467644101</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>13</v>
       </c>
@@ -40469,7 +40466,7 @@
         <v>0.24956114314017558</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>13</v>
       </c>
@@ -40501,7 +40498,7 @@
         <v>0.11472538235515707</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>13</v>
       </c>
@@ -40533,7 +40530,7 @@
         <v>0.11066783056409726</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>13</v>
       </c>
@@ -40565,7 +40562,7 @@
         <v>3.1019766549647242E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>13</v>
       </c>
@@ -40597,7 +40594,7 @@
         <v>2.5573439562543449E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>13</v>
       </c>
@@ -40629,7 +40626,7 @@
         <v>1.3918787547388725E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>13</v>
       </c>
@@ -40661,7 +40658,7 @@
         <v>7.1168181711962226E-3</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>13</v>
       </c>
@@ -40693,7 +40690,7 @@
         <v>1.9343362651094813E-3</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>13</v>
       </c>
@@ -40725,7 +40722,7 @@
         <v>1.548754237567209E-3</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>13</v>
       </c>
@@ -40757,7 +40754,7 @@
         <v>1.3795664532925138E-3</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>14</v>
       </c>
@@ -40789,7 +40786,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>14</v>
       </c>
@@ -40821,7 +40818,7 @@
         <v>0.46948723310332008</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>14</v>
       </c>
@@ -40853,7 +40850,7 @@
         <v>0.19647635345364031</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>14</v>
       </c>
@@ -40885,7 +40882,7 @@
         <v>0.13493163673854225</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>14</v>
       </c>
@@ -40917,7 +40914,7 @@
         <v>9.5209556010388274E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>14</v>
       </c>
@@ -40949,7 +40946,7 @@
         <v>7.2108309484216773E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>14</v>
       </c>
@@ -40981,7 +40978,7 @@
         <v>5.6228761727310873E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>13</v>
       </c>
@@ -41013,7 +41010,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>13</v>
       </c>
@@ -41045,7 +41042,7 @@
         <v>0.99984463330734807</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>13</v>
       </c>
@@ -41077,7 +41074,7 @@
         <v>0.49855704235816883</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>13</v>
       </c>
@@ -41109,7 +41106,7 @@
         <v>0.10368646530339042</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>13</v>
       </c>
@@ -41141,7 +41138,7 @@
         <v>0.11219493445607351</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>13</v>
       </c>
@@ -41173,7 +41170,7 @@
         <v>3.7706125145366073E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>13</v>
       </c>
@@ -41205,7 +41202,7 @@
         <v>2.6156598601813481E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>13</v>
       </c>
@@ -41237,7 +41234,7 @@
         <v>1.0306267778518194E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>13</v>
       </c>
@@ -41269,7 +41266,7 @@
         <v>6.2621877672431516E-3</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>13</v>
       </c>
@@ -41301,7 +41298,7 @@
         <v>1.8947856716542745E-3</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>13</v>
       </c>
@@ -41333,7 +41330,7 @@
         <v>1.4363648740264578E-3</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>13</v>
       </c>
@@ -41365,7 +41362,7 @@
         <v>8.0077196894524937E-4</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>14</v>
       </c>
@@ -41397,7 +41394,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>14</v>
       </c>
@@ -41429,7 +41426,7 @@
         <v>0.88535384765412894</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>14</v>
       </c>
@@ -41461,7 +41458,7 @@
         <v>0.3653931642851001</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>14</v>
       </c>
@@ -41493,7 +41490,7 @@
         <v>0.23864467978209061</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>14</v>
       </c>
@@ -41525,7 +41522,7 @@
         <v>0.16988155423703441</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>14</v>
       </c>
@@ -41557,7 +41554,7 @@
         <v>0.1307385418984906</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>14</v>
       </c>
@@ -41589,7 +41586,7 @@
         <v>0.10201471066689344</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>13</v>
       </c>
@@ -41621,7 +41618,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>13</v>
       </c>
@@ -41653,7 +41650,7 @@
         <v>0.99654901186076605</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>13</v>
       </c>
@@ -41685,7 +41682,7 @@
         <v>0.98543159897951638</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>13</v>
       </c>
@@ -41717,7 +41714,7 @@
         <v>0.3684713355428228</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>13</v>
       </c>
@@ -41749,7 +41746,7 @@
         <v>0.45585268215571889</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>13</v>
       </c>
@@ -41781,7 +41778,7 @@
         <v>0.2155209609486631</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>13</v>
       </c>
@@ -41813,7 +41810,7 @@
         <v>0.1702707127363623</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>13</v>
       </c>
@@ -41845,7 +41842,7 @@
         <v>9.0960496590248817E-3</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>13</v>
       </c>
@@ -41877,7 +41874,7 @@
         <v>4.1466759143931348E-3</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>13</v>
       </c>
@@ -41909,7 +41906,7 @@
         <v>2.0522314405363802E-3</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>13</v>
       </c>
@@ -41941,7 +41938,7 @@
         <v>6.3901341438181946E-4</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>13</v>
       </c>
@@ -41973,7 +41970,7 @@
         <v>6.6694420296401619E-4</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>14</v>
       </c>
@@ -42005,7 +42002,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>14</v>
       </c>
@@ -42037,7 +42034,7 @@
         <v>0.94041209437758422</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>14</v>
       </c>
@@ -42069,7 +42066,7 @@
         <v>0.68224686836460302</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>14</v>
       </c>
@@ -42101,7 +42098,7 @@
         <v>0.65807486898674072</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>14</v>
       </c>
@@ -42133,7 +42130,7 @@
         <v>0.60680636281346589</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>14</v>
       </c>
@@ -42165,7 +42162,7 @@
         <v>0.55663318435868636</v>
       </c>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>14</v>
       </c>
@@ -42197,7 +42194,7 @@
         <v>0.47856897959710848</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>13</v>
       </c>
@@ -42229,7 +42226,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>13</v>
       </c>
@@ -42261,7 +42258,7 @@
         <v>0.99756444619022311</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>13</v>
       </c>
@@ -42293,7 +42290,7 @@
         <v>0.99532565641160808</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>13</v>
       </c>
@@ -42325,7 +42322,7 @@
         <v>0.45906153834138252</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>13</v>
       </c>
@@ -42357,7 +42354,7 @@
         <v>0.46622912352339241</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>13</v>
       </c>
@@ -42389,7 +42386,7 @@
         <v>0.29359654178347722</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>13</v>
       </c>
@@ -42421,7 +42418,7 @@
         <v>0.2887834756729471</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>13</v>
       </c>
@@ -42453,7 +42450,7 @@
         <v>0.20722359640589069</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>13</v>
       </c>
@@ -42485,7 +42482,7 @@
         <v>0.12550120449373128</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>13</v>
       </c>
@@ -42517,7 +42514,7 @@
         <v>6.6500541366207977E-2</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>13</v>
       </c>
@@ -42549,7 +42546,7 @@
         <v>7.9099132110241624E-2</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>13</v>
       </c>
@@ -42581,7 +42578,7 @@
         <v>4.0166972152507266E-2</v>
       </c>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>14</v>
       </c>
@@ -42613,7 +42610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>14</v>
       </c>
@@ -42645,7 +42642,7 @@
         <v>0.93262544044482731</v>
       </c>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>14</v>
       </c>
@@ -42677,7 +42674,7 @@
         <v>0.69945710865242472</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>14</v>
       </c>
@@ -42709,7 +42706,7 @@
         <v>0.6165005335141226</v>
       </c>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>14</v>
       </c>
@@ -42741,7 +42738,7 @@
         <v>0.57315526949210616</v>
       </c>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>14</v>
       </c>
@@ -42773,7 +42770,7 @@
         <v>0.52945564614768181</v>
       </c>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>14</v>
       </c>
@@ -42805,7 +42802,7 @@
         <v>0.44167756907735806</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>13</v>
       </c>
@@ -42837,7 +42834,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>13</v>
       </c>
@@ -42869,7 +42866,7 @@
         <v>0.99814488127085876</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>13</v>
       </c>
@@ -42901,7 +42898,7 @@
         <v>0.99624812044725419</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>13</v>
       </c>
@@ -42933,7 +42930,7 @@
         <v>0.99691659673129307</v>
       </c>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>13</v>
       </c>
@@ -42965,7 +42962,7 @@
         <v>0.99441501861107306</v>
       </c>
     </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>13</v>
       </c>
@@ -42997,7 +42994,7 @@
         <v>0.99143396170539866</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>13</v>
       </c>
@@ -43029,7 +43026,7 @@
         <v>0.99087686513722062</v>
       </c>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>13</v>
       </c>
@@ -43061,7 +43058,7 @@
         <v>0.98926966722020515</v>
       </c>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>13</v>
       </c>
@@ -43093,7 +43090,7 @@
         <v>0.98484015102390055</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>13</v>
       </c>
@@ -43125,7 +43122,7 @@
         <v>0.98284384903777278</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>13</v>
       </c>
@@ -43157,7 +43154,7 @@
         <v>0.98514403679262685</v>
       </c>
     </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>13</v>
       </c>
@@ -43189,7 +43186,7 @@
         <v>0.98228240229147923</v>
       </c>
     </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>14</v>
       </c>
@@ -43221,7 +43218,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>14</v>
       </c>
@@ -43253,7 +43250,7 @@
         <v>0.9472980047936107</v>
       </c>
     </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>14</v>
       </c>
@@ -43285,7 +43282,7 @@
         <v>0.72660128045650318</v>
       </c>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>14</v>
       </c>
@@ -43317,7 +43314,7 @@
         <v>0.66059890031419355</v>
       </c>
     </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>14</v>
       </c>
@@ -43349,7 +43346,7 @@
         <v>0.60934001918612435</v>
       </c>
     </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>14</v>
       </c>
@@ -43381,7 +43378,7 @@
         <v>0.57706889753863133</v>
       </c>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>14</v>
       </c>
@@ -43413,7 +43410,7 @@
         <v>0.49049005627738529</v>
       </c>
     </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>13</v>
       </c>
@@ -43445,7 +43442,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>13</v>
       </c>
@@ -43477,7 +43474,7 @@
         <v>0.99944317456377119</v>
       </c>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>13</v>
       </c>
@@ -43509,7 +43506,7 @@
         <v>0.99813285421281028</v>
       </c>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>13</v>
       </c>
@@ -43541,7 +43538,7 @@
         <v>0.99846230909790246</v>
       </c>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>13</v>
       </c>
@@ -43573,7 +43570,7 @@
         <v>0.99775084449779505</v>
       </c>
     </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>13</v>
       </c>
@@ -43605,7 +43602,7 @@
         <v>0.99676012420954696</v>
       </c>
     </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>13</v>
       </c>
@@ -43637,7 +43634,7 @@
         <v>0.99507500392366433</v>
       </c>
     </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>13</v>
       </c>
@@ -43669,7 +43666,7 @@
         <v>0.9942673044763769</v>
       </c>
     </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>13</v>
       </c>
@@ -43701,7 +43698,7 @@
         <v>0.99436825673670659</v>
       </c>
     </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>13</v>
       </c>
@@ -43733,7 +43730,7 @@
         <v>0.99303666633845866</v>
       </c>
     </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>13</v>
       </c>
@@ -43765,7 +43762,7 @@
         <v>0.99326566288921936</v>
       </c>
     </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>13</v>
       </c>
@@ -43797,7 +43794,7 @@
         <v>0.99114727756458465</v>
       </c>
     </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>14</v>
       </c>
@@ -43829,7 +43826,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>14</v>
       </c>
@@ -43861,7 +43858,7 @@
         <v>1.3342843672428888</v>
       </c>
     </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>14</v>
       </c>
@@ -43893,7 +43890,7 @@
         <v>1.2749982143979377</v>
       </c>
     </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>14</v>
       </c>
@@ -43925,7 +43922,7 @@
         <v>1.111125387497683</v>
       </c>
     </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>14</v>
       </c>
@@ -43957,7 +43954,7 @@
         <v>0.99348249233467512</v>
       </c>
     </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>14</v>
       </c>
@@ -43989,7 +43986,7 @@
         <v>0.96664497809397376</v>
       </c>
     </row>
-    <row r="153" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>14</v>
       </c>
@@ -44021,7 +44018,7 @@
         <v>0.86385795894476647</v>
       </c>
     </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>13</v>
       </c>
@@ -44053,7 +44050,7 @@
         <v>3.1420481759501531E-2</v>
       </c>
     </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>13</v>
       </c>
@@ -44085,7 +44082,7 @@
         <v>3.121294685564668E-2</v>
       </c>
     </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>13</v>
       </c>
@@ -44117,7 +44114,7 @@
         <v>3.125E-2</v>
       </c>
     </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>14</v>
       </c>
@@ -44149,7 +44146,7 @@
         <v>0.19451466517209187</v>
       </c>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>14</v>
       </c>
@@ -44181,7 +44178,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>14</v>
       </c>
@@ -44213,7 +44210,7 @@
         <v>7.6377886833008529E-2</v>
       </c>
     </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>13</v>
       </c>
@@ -44245,7 +44242,7 @@
         <v>3.1421721251165248E-2</v>
       </c>
     </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>13</v>
       </c>
@@ -44277,7 +44274,7 @@
         <v>3.1266157054522938E-2</v>
       </c>
     </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>13</v>
       </c>
@@ -44321,21 +44318,22 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A82197F5-6B8C-46C5-BB99-B49F4017F852}">
+  <sheetPr codeName="Foglio2"/>
   <dimension ref="A1:N12"/>
-  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.75" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.625" customWidth="1"/>
-    <col min="10" max="10" width="15.75" customWidth="1"/>
+    <col min="4" max="4" width="18.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.6640625" customWidth="1"/>
+    <col min="10" max="10" width="15.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -44373,7 +44371,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -44419,7 +44417,7 @@
         <v>0.25303798733636451</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -44465,7 +44463,7 @@
         <v>9.5064926616680159E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -44511,7 +44509,7 @@
         <v>6.204639921747768E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -44546,7 +44544,7 @@
         <v>9.5064926616680159E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -44581,7 +44579,7 @@
         <v>7.1778666328254767E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -44616,7 +44614,7 @@
         <v>6.3591085000199665E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -44651,7 +44649,7 @@
         <v>5.3361452410325971E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -44686,7 +44684,7 @@
         <v>3.8767859774241069E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -44721,7 +44719,7 @@
         <v>2.7308898109650731E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -44756,7 +44754,7 @@
         <v>6.204639921747768E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>14</v>
       </c>

</xml_diff>